<commit_message>
BI data sync 2026-09-19 11:01:26
</commit_message>
<xml_diff>
--- a/Master_Settings.xlsx
+++ b/Master_Settings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\OPERATION\Delivery Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F909C38A-BFC4-40C1-8C57-A197FF19624E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C302ADFA-107F-4D92-9C5A-15FEC69ADD4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{CC1BE0F9-419A-45B7-A77C-3F121AEBD672}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CC1BE0F9-419A-45B7-A77C-3F121AEBD672}"/>
   </bookViews>
   <sheets>
     <sheet name="Drivers" sheetId="1" r:id="rId1"/>
@@ -10672,30 +10672,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>3387</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C2" s="4">
-        <v>35</v>
-      </c>
-      <c r="D2" s="3">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="D2" s="5">
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>3388</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C3" s="4">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3">
-        <v>30</v>
+        <v>18</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -10703,10 +10703,10 @@
         <v>34</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C4" s="4">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="D4" s="3">
         <v>20</v>
@@ -10714,27 +10714,27 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D5" s="3">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" s="4">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D6" s="3">
         <v>20</v>
@@ -10742,13 +10742,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D7" s="3">
         <v>20</v>
@@ -10756,44 +10756,44 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C8" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D8" s="3">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C9" s="4">
-        <v>15</v>
-      </c>
-      <c r="D9" s="5">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="D9" s="3">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="4">
         <v>15</v>
       </c>
-      <c r="C10" s="4">
-        <v>20</v>
-      </c>
-      <c r="D10" s="5">
-        <v>40</v>
+      <c r="D10" s="3">
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -10801,38 +10801,38 @@
         <v>14</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="4">
-        <v>10</v>
-      </c>
-      <c r="D11" s="3">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C12" s="4">
-        <v>24</v>
-      </c>
-      <c r="D12" s="3">
         <v>20</v>
+      </c>
+      <c r="D12" s="5">
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C13" s="4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D13" s="3">
         <v>30</v>
@@ -10840,27 +10840,27 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C14" s="4">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="D14" s="3">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3">
         <v>30</v>
@@ -10868,41 +10868,41 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C16" s="4">
-        <v>30</v>
-      </c>
-      <c r="D16" s="5">
-        <v>20</v>
+        <v>44</v>
+      </c>
+      <c r="D16" s="3">
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" s="4">
-        <v>20</v>
-      </c>
-      <c r="D17" s="5">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="D17" s="3">
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C18" s="4">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D18" s="5">
         <v>20</v>
@@ -10910,57 +10910,57 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C19" s="4">
-        <v>10</v>
-      </c>
-      <c r="D19" s="3">
-        <v>30</v>
+        <v>20</v>
+      </c>
+      <c r="D19" s="5">
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C20" s="4">
-        <v>32</v>
-      </c>
-      <c r="D20" s="3">
+        <v>28</v>
+      </c>
+      <c r="D20" s="5">
         <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C21" s="4">
-        <v>52</v>
-      </c>
-      <c r="D21" s="5">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="D21" s="3">
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="4">
-        <v>16</v>
-      </c>
-      <c r="D22" s="5">
+        <v>32</v>
+      </c>
+      <c r="D22" s="3">
         <v>20</v>
       </c>
     </row>
@@ -10969,66 +10969,66 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C23" s="4">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="D23" s="5">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C24" s="4">
-        <v>20</v>
-      </c>
-      <c r="D24" s="3">
+        <v>16</v>
+      </c>
+      <c r="D24" s="5">
         <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C25" s="4">
-        <v>36</v>
-      </c>
-      <c r="D25" s="3">
-        <v>10</v>
+        <v>22</v>
+      </c>
+      <c r="D25" s="5">
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C26" s="4">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D26" s="3">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C27" s="4">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D27" s="3">
         <v>10</v>
@@ -11036,83 +11036,83 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C28" s="4">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D28" s="3">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C29" s="4">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="D29" s="3">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C30" s="4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D30" s="3">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="C31" s="4">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D31" s="3">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="4">
-        <v>19</v>
-      </c>
-      <c r="D32" s="5">
-        <v>1</v>
+        <v>28</v>
+      </c>
+      <c r="D32" s="3">
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C33" s="4">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="D33" s="3">
         <v>20</v>
@@ -11120,35 +11120,35 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C34" s="4">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D34" s="5">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C35" s="4">
-        <v>20</v>
-      </c>
-      <c r="D35" s="5">
+        <v>19</v>
+      </c>
+      <c r="D35" s="3">
         <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>10</v>
@@ -11156,145 +11156,145 @@
       <c r="C36" s="4">
         <v>12</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="5">
         <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C37" s="4">
         <v>20</v>
       </c>
-      <c r="D37" s="3">
-        <v>30</v>
+      <c r="D37" s="5">
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C38" s="4">
-        <v>24</v>
-      </c>
-      <c r="D38" s="5">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="D38" s="3">
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="C39" s="4">
-        <v>48</v>
-      </c>
-      <c r="D39" s="5">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="D39" s="3">
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C40" s="4">
-        <v>34</v>
-      </c>
-      <c r="D40" s="3">
-        <v>10</v>
+        <v>24</v>
+      </c>
+      <c r="D40" s="5">
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C41" s="4">
-        <v>18</v>
-      </c>
-      <c r="D41" s="3">
-        <v>20</v>
+        <v>48</v>
+      </c>
+      <c r="D41" s="5">
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" s="4">
+        <v>34</v>
+      </c>
+      <c r="D42" s="3">
         <v>10</v>
-      </c>
-      <c r="C42" s="4">
-        <v>12</v>
-      </c>
-      <c r="D42" s="3">
-        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="C43" s="4">
-        <v>34</v>
-      </c>
-      <c r="D43" s="5">
-        <v>10</v>
+        <v>18</v>
+      </c>
+      <c r="D43" s="3">
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C44" s="4">
-        <v>30</v>
-      </c>
-      <c r="D44" s="5">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="D44" s="3">
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C45" s="4">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="D45" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>3385</v>
+        <v>37</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C46" s="4">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D46" s="5">
         <v>10</v>
@@ -11302,63 +11302,63 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>3386</v>
+        <v>37</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C47" s="4">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D47" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>3386</v>
+        <v>3385</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C48" s="4">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D48" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>48</v>
+        <v>3386</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C49" s="4">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D49" s="5">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>49</v>
+        <v>3386</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C50" s="4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D50" s="5">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>41</v>
@@ -11372,13 +11372,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C52" s="4">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D52" s="5">
         <v>1</v>
@@ -11386,13 +11386,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C53" s="4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D53" s="5">
         <v>1</v>
@@ -11400,13 +11400,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C54" s="4">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D54" s="5">
         <v>1</v>
@@ -11414,13 +11414,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C55" s="4">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D55" s="5">
         <v>1</v>
@@ -11428,7 +11428,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>41</v>
@@ -11442,13 +11442,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C57" s="4">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D57" s="5">
         <v>1</v>
@@ -11456,13 +11456,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C58" s="4">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D58" s="5">
         <v>1</v>
@@ -11470,13 +11470,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C59" s="4">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D59" s="5">
         <v>1</v>
@@ -11484,13 +11484,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C60" s="4">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D60" s="5">
         <v>1</v>
@@ -11498,13 +11498,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C61" s="4">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D61" s="5">
         <v>1</v>
@@ -11512,13 +11512,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C62" s="4">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D62" s="5">
         <v>1</v>
@@ -11526,13 +11526,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C63" s="4">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D63" s="5">
         <v>1</v>
@@ -11540,7 +11540,7 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>3389</v>
+        <v>61</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>41</v>
@@ -11554,13 +11554,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>3390</v>
+        <v>62</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>41</v>
       </c>
       <c r="C65" s="4">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D65" s="5">
         <v>1</v>
@@ -11568,27 +11568,27 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>3387</v>
+        <v>3389</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C66" s="4">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D66" s="5">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>3388</v>
+        <v>3390</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C67" s="4">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D67" s="5">
         <v>1</v>

</xml_diff>

<commit_message>
BI data sync 2026-10-12 10:01:17
</commit_message>
<xml_diff>
--- a/Master_Settings.xlsx
+++ b/Master_Settings.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\OPERATION\Delivery Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\OPERATION\Delivery Plan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C302ADFA-107F-4D92-9C5A-15FEC69ADD4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AD9787D-6009-469C-AA53-94A6A3E7D80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{CC1BE0F9-419A-45B7-A77C-3F121AEBD672}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{CC1BE0F9-419A-45B7-A77C-3F121AEBD672}"/>
   </bookViews>
   <sheets>
     <sheet name="Drivers" sheetId="1" r:id="rId1"/>
     <sheet name="Inventory" sheetId="2" r:id="rId2"/>
-    <sheet name="Debtor Code" sheetId="4" r:id="rId3"/>
+    <sheet name="ItemCode" sheetId="5" r:id="rId3"/>
+    <sheet name="Debtor Code" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4323" uniqueCount="3391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4512" uniqueCount="3580">
   <si>
     <t>Driver Name</t>
   </si>
@@ -10200,6 +10201,573 @@
   </si>
   <si>
     <t>PSIKOLOGI</t>
+  </si>
+  <si>
+    <t>BR964S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Rujukan Biologi STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLO16R</t>
+  </si>
+  <si>
+    <t>BR964S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Rujukan Biologi STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLO26R</t>
+  </si>
+  <si>
+    <t>BR964S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Reference Exercise Biology STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLO36R</t>
+  </si>
+  <si>
+    <t>BR922S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Rujukan Kesusasteraan Melayu Komunikatif STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLK26R</t>
+  </si>
+  <si>
+    <t>BR922S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Rujukan Kesusateraan Melayu Komunikatif STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLK16R</t>
+  </si>
+  <si>
+    <t>BR80026</t>
+  </si>
+  <si>
+    <t>LPS1 : Thematic Muet 2026</t>
+  </si>
+  <si>
+    <t>KLM16R</t>
+  </si>
+  <si>
+    <t>BR948S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Rujukan Perakaunan STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLN16R</t>
+  </si>
+  <si>
+    <t>NL900S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Minda &amp; Lembaran Praktis Pengajian Am STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLA16L</t>
+  </si>
+  <si>
+    <t>BR948S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Rujukan Perakaunan STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLN36R</t>
+  </si>
+  <si>
+    <t>NL900S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Minda &amp; Lembaran Praktis Pengajian Am STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLA26L</t>
+  </si>
+  <si>
+    <t>BR970S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Rujukan Lukisan Seni Visual STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLV16R</t>
+  </si>
+  <si>
+    <t>BR944S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Rujukan Ekonomi STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLE36R</t>
+  </si>
+  <si>
+    <t>NL913S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Pembelajaran &amp; Lembaran Praktis Bahasa Arab STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLR16L</t>
+  </si>
+  <si>
+    <t>NL900S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Nota Minda &amp; Lembaran Praktis Pengajian Am STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLA36L</t>
+  </si>
+  <si>
+    <t>NL966S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Modul Sains Sukan STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLS36L</t>
+  </si>
+  <si>
+    <t>NL930S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Pembelajaran &amp; Lembaran Praktis Pengajian Syariah Kontemporari STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLY16L</t>
+  </si>
+  <si>
+    <t>BR970S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Rujukan Seni Visual STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLV26R</t>
+  </si>
+  <si>
+    <t>ESEI90026</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Penulisan Esei Pengajian Am STPM (2026)</t>
+  </si>
+  <si>
+    <t>KLA16E</t>
+  </si>
+  <si>
+    <t>MTP80026</t>
+  </si>
+  <si>
+    <t>LPS1 : Muet Test Paper (2026)</t>
+  </si>
+  <si>
+    <t>KLM16M</t>
+  </si>
+  <si>
+    <t>BR948S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Rujukan Perakauanan STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLN26R</t>
+  </si>
+  <si>
+    <t>EP964S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Topical Exercise Biology STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLO36L</t>
+  </si>
+  <si>
+    <t>MTP964S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Biologi STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLO26M</t>
+  </si>
+  <si>
+    <t>NL942S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Pembelajaran &amp; Lembaran Praktis Geografi STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLG16L</t>
+  </si>
+  <si>
+    <t>NL946AS226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Pembelajaran &amp; Lembaran Praktis Pengajian Perniagaan STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLP26N</t>
+  </si>
+  <si>
+    <t>NL946BS226</t>
+  </si>
+  <si>
+    <t>LPS2 : Modul Pengajian Perniagaan STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLP26L</t>
+  </si>
+  <si>
+    <t>NL942S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Pembelajaran &amp; Lembaran Praktis Geografi STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLG26L</t>
+  </si>
+  <si>
+    <t>NL940S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Modul Sejarah STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLJ36L</t>
+  </si>
+  <si>
+    <t>NL970S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Lembaran Praktis Seni Visual STPM Semester2 (2026)</t>
+  </si>
+  <si>
+    <t>KLV26L</t>
+  </si>
+  <si>
+    <t>NL931S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Pembelajaran &amp; Lembaran Praktis Pengajian Usuluddin STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLU16L</t>
+  </si>
+  <si>
+    <t>NL913S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Nota Pembelajaran &amp; Lembaran Praktis Bahasa Arab STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLR36L</t>
+  </si>
+  <si>
+    <t>NL946BS126</t>
+  </si>
+  <si>
+    <t>LPS1 : Modul Pengajian Perniagaan STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLP16L</t>
+  </si>
+  <si>
+    <t>NL944S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Pembelajaran &amp; Lembaran Praktis Ekonomi STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLE26L</t>
+  </si>
+  <si>
+    <t>EP962S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Topical Exercises Chemistry STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLC16L</t>
+  </si>
+  <si>
+    <t>NL946BS326</t>
+  </si>
+  <si>
+    <t>LPS3 : Modul Pengajian Perniagaan STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLP36L</t>
+  </si>
+  <si>
+    <t>BR922S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Rujukan Kesusasteraan Melayu Komunikatif STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLK36R</t>
+  </si>
+  <si>
+    <t>NL931S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Pembelajaran &amp; Lembaran Praktis Usuluddin STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLU26L</t>
+  </si>
+  <si>
+    <t>NL913S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Pembelajaran &amp; Lembaran Praktis Bahasa Arab STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLR26L</t>
+  </si>
+  <si>
+    <t>NL910S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Nota Pembelajaran &amp; Lembaran Praktis Bahasa Melayu STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLB36L</t>
+  </si>
+  <si>
+    <t>NL910S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Nota Pembelajaran &amp; Lembaran Praktis Bahasa Melayu STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLB16L</t>
+  </si>
+  <si>
+    <t>EP964S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Topical &amp; Exercise Biology STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLO26L</t>
+  </si>
+  <si>
+    <t>MTP940S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Sejarah STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLJ26M</t>
+  </si>
+  <si>
+    <t>MTP900S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Model Kertas Peperiksaan Pengajian Am STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLA36M</t>
+  </si>
+  <si>
+    <t>MTP940S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Kertas Model Peperiksaan Sejarah STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLJ36M</t>
+  </si>
+  <si>
+    <t>MTP922S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Model Kertas Peperiksaan Kesusasteraan Melayu Komunikatif STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLK36M</t>
+  </si>
+  <si>
+    <t>MTP922S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Kesusasteraan Melayu Komunakatif STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLK26M</t>
+  </si>
+  <si>
+    <t>MTP922S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Kesusasteraan Melayu Komunikatif STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLK16M</t>
+  </si>
+  <si>
+    <t>MTP910S326</t>
+  </si>
+  <si>
+    <t>LPS3 : Model Kertas Peperiksaan Bahasa Melayu STPM Semester 3 (2026)</t>
+  </si>
+  <si>
+    <t>KLB36M</t>
+  </si>
+  <si>
+    <t>MTP910S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Bahasa Melayu STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLB26M</t>
+  </si>
+  <si>
+    <t>NL910S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Nota Padat &amp; Lembaran Praktis Bahasa Melayu STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLB26L</t>
+  </si>
+  <si>
+    <t>MTP910S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Bahasa Melayu STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLB16M</t>
+  </si>
+  <si>
+    <t>MTP900S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Pengajian Am STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLA26M</t>
+  </si>
+  <si>
+    <t>MTP900S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Pengajian Am STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLA16M</t>
+  </si>
+  <si>
+    <t>MTP942S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Geografi STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLG16M</t>
+  </si>
+  <si>
+    <t>MTP946S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Pengajian Perniagaan STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLP16M</t>
+  </si>
+  <si>
+    <t>MTP946S226</t>
+  </si>
+  <si>
+    <t>LPS2 : Model Kertas Peperiksaan Pengajian Perniagaan STPM Semester 2 (2026)</t>
+  </si>
+  <si>
+    <t>KLP26M</t>
+  </si>
+  <si>
+    <t>MTP940S126</t>
+  </si>
+  <si>
+    <t>LPS1 : Model Kertas Peperiksaan Sejarah STPM Semester 1 (2026)</t>
+  </si>
+  <si>
+    <t>KLJ16M</t>
+  </si>
+  <si>
+    <t>Description2</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Item Code</t>
+  </si>
+  <si>
+    <t>NLLKT426</t>
+  </si>
+  <si>
+    <t>LP4 : Lembaran Praktis Lukisan Kejuruteraan T4 (2026)</t>
+  </si>
+  <si>
+    <t>KL6T4NL</t>
+  </si>
+  <si>
+    <t>NLLKT525</t>
+  </si>
+  <si>
+    <t>LP5 : Lembaran Praktis Lukisan Kejuruteraan T5 (2025)</t>
+  </si>
+  <si>
+    <t>KL5T5NL</t>
+  </si>
+  <si>
+    <t>MTPLKSPM25</t>
+  </si>
+  <si>
+    <t>LP5 : MTP Lukisan Kejuruteraan SPM (2025)</t>
+  </si>
+  <si>
+    <t>KL5T5ML</t>
+  </si>
+  <si>
+    <t>NLGKTT426</t>
+  </si>
+  <si>
+    <t>LP4 : Lembaran Praktis Grafik Komunikasi Teknikal T4 (2026)</t>
+  </si>
+  <si>
+    <t>KL6T4NT</t>
+  </si>
+  <si>
+    <t>NLGKTT525</t>
+  </si>
+  <si>
+    <t>LP5 : Lembaran Praktis Grafik Komunikasi Teknikal T5 (2025)</t>
+  </si>
+  <si>
+    <t>KL5T5NT</t>
+  </si>
+  <si>
+    <t>MTPGKTSPM25</t>
+  </si>
+  <si>
+    <t>LP5 : MTP Grafik Komunikasi Teknikal SPM (2025)</t>
+  </si>
+  <si>
+    <t>KL5T5MT</t>
   </si>
 </sst>
 </file>
@@ -10209,7 +10777,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;RM&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -10230,16 +10798,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -10262,11 +10845,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFA9A9A9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFA9A9A9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFA9A9A9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFA9A9A9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -10285,6 +10883,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11600,6 +12204,714 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA081120-94CF-4E97-87C5-7879CDD64AE9}">
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="74" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>3561</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>3560</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>3559</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>3558</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>3557</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>3556</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>3555</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>3554</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>3553</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>3552</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>3551</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>3550</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>3549</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>3548</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>3547</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>3546</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>3545</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>3544</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>3543</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>3542</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>3541</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>3540</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>3539</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>3538</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>3537</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>3536</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>3535</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>3534</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>3533</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>3532</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>3531</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>3530</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>3529</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>3528</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>3527</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>3526</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>3525</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>3524</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>3523</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>3522</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>3521</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>3520</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>3519</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>3518</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>3517</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>3516</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>3515</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>3514</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>3513</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>3512</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>3511</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>3510</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>3509</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>3508</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>3507</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>3506</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>3505</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>3504</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>3503</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>3502</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>3501</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>3500</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>3499</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>3498</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>3497</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>3496</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>3495</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>3494</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>3493</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>3492</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>3491</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>3490</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>3489</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>3488</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>3487</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>3486</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>3485</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>3484</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>3483</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>3482</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>3481</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>3480</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>3479</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>3478</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>3477</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>3476</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>3475</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>3474</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>3473</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>3472</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>3471</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>3470</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>3469</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>3468</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>3467</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>3466</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>3465</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>3464</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>3463</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>3462</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>3461</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>3460</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>3459</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>3458</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>3457</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>3456</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>3455</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>3454</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>3453</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>3452</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>3451</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="7" t="s">
+        <v>3450</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>3449</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>3448</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>3447</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>3446</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>3445</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>3444</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>3443</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>3442</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>3441</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>3440</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>3439</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="7" t="s">
+        <v>3438</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>3437</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>3436</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>3435</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>3434</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>3433</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>3432</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>3431</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>3430</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
+        <v>3429</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>3428</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>3427</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="7" t="s">
+        <v>3426</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>3425</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>3424</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>3423</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>3422</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>3421</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
+        <v>3420</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>3419</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>3418</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="7" t="s">
+        <v>3417</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>3416</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>3415</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="7" t="s">
+        <v>3414</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>3413</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>3412</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="7" t="s">
+        <v>3411</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>3410</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>3409</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="7" t="s">
+        <v>3408</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>3407</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>3406</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="7" t="s">
+        <v>3405</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>3404</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>3403</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="7" t="s">
+        <v>3402</v>
+      </c>
+      <c r="B54" s="7" t="s">
+        <v>3401</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="7" t="s">
+        <v>3399</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>3398</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>3397</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="7" t="s">
+        <v>3396</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>3395</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>3394</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>3393</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>3392</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>3391</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>3570</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>3569</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>3568</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
+        <v>3567</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>3566</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>3565</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="7" t="s">
+        <v>3564</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>3563</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>3562</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
+        <v>3579</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>3578</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>3577</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
+        <v>3576</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>3575</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>3574</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>3573</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>3572</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>3571</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B9E555B-0667-40CE-8431-15EDC2CA6AFC}">
   <dimension ref="A1:C1393"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>